<commit_message>
11.09.2026 - PCB design and schematics changes
</commit_message>
<xml_diff>
--- a/Keyboard BOM.xlsx
+++ b/Keyboard BOM.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/5ac8f2ab3c324b6b/Documents/GitHub/Crazy-75/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="119" documentId="8_{FCCC2E56-FDB1-4E02-ACF6-F81B5EFE9B54}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{8F25B597-E420-475F-8842-6639776565E0}"/>
+  <xr:revisionPtr revIDLastSave="137" documentId="8_{FCCC2E56-FDB1-4E02-ACF6-F81B5EFE9B54}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{57AED7F5-C1AE-439E-BAFC-F0568EF62BD8}"/>
   <bookViews>
-    <workbookView xWindow="11145" yWindow="4920" windowWidth="27300" windowHeight="15300" xr2:uid="{7E7D5457-AF9F-4A24-AB89-FCDAB66E2EA5}"/>
+    <workbookView xWindow="24045" yWindow="4665" windowWidth="27300" windowHeight="15300" xr2:uid="{7E7D5457-AF9F-4A24-AB89-FCDAB66E2EA5}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="41" uniqueCount="31">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="44" uniqueCount="34">
   <si>
     <t>Part No.</t>
   </si>
@@ -92,15 +92,6 @@
     <t>EC11</t>
   </si>
   <si>
-    <t>https://fr.aliexpress.com/item/1005007369669431.html?spm=a2g0o.productlist.main.3.193201TR01TR1P&amp;algo_pvid=1936a5f8-4955-4ddf-ab19-5181f7e135f5&amp;algo_exp_id=1936a5f8-4955-4ddf-ab19-5181f7e135f5-2&amp;pdp_ext_f=%7B%22order%22%3A%22764%22%2C%22spu_best_type%22%3A%22price%22%2C%22eval%22%3A%221%22%2C%22fromPage%22%3A%22search%22%7D&amp;pdp_npi=6%40dis%21EUR%212.75%212.75%21%21%213.14%213.14%21%400be71e1e17877677506374984e0f30%2112000040462155655%21sea%21LU%218155715332%21X%211%210%21n_tag%3A-29911%3Bd%3Ae8fc6401%3Bm03_new_user%3A-29895&amp;curPageLogUid=LZYu56IlV2lS&amp;utparam-url=scene%3Asearch%7Cquery_from%3A%7Cx_object_id%3A1005007369669431%7C_p_origin_prod%3A</t>
-  </si>
-  <si>
-    <t>RP2040 Raspberry Pi Pico-compatible, standard 40-pin / 21 × 51 mm footprint</t>
-  </si>
-  <si>
-    <t>Pico clone</t>
-  </si>
-  <si>
     <t>Switches</t>
   </si>
   <si>
@@ -132,19 +123,43 @@
   </si>
   <si>
     <t>6.25u &amp; 3x2u</t>
+  </si>
+  <si>
+    <t>Fine tweezers</t>
+  </si>
+  <si>
+    <t>https://fr.aliexpress.com/item/1005005589349988.html?spm=a2g0n.productlist.0.0.659b7Fq27Fq2R9&amp;browser_id=2269fcae49994bc495ac18d9a18a9643&amp;aff_trace_key=a9b6c8e739aa4a98a2d8e403b501ff28-1780918887469-07997-_DFhInr9&amp;aff_platform=msite&amp;m_page_id=v5mtilbuikgcav781a084e0c4411236e9b8532da4f&amp;gclid=&amp;pdp_ext_f=%7B%22order%22%3A%228727%22%2C%22spu_best_type%22%3A%22price%22%2C%22eval%22%3A%221%22%2C%22fromPage%22%3A%22search%22%7D&amp;pdp_npi=6%40dis%21EUR%211.73%211.73%21%21%2113.19%2113.19%21%40ac1030a317889357179444389d6200%2112000033663600866%21sea%21LU%218155715332%21X%211%210%21n_tag%3A-29911%3Bd%3A5b165265%3Bm03_new_user%3A-29895&amp;algo_pvid=fe0d1407-89bd-480f-8040-2026dc62325d&amp;utparam-url=scene%3Asearch%7Cquery_from%3A%7Cx_object_id%3A1005005589349988%7C_p_origin_prod%3A</t>
+  </si>
+  <si>
+    <t>straight and curved fine tweezers</t>
+  </si>
+  <si>
+    <t>https://fr.aliexpress.com/item/1005006967374887.html?spm=a2g0o.productlist.main.2.54a5NjX2NjX24Z&amp;algo_pvid=b81f8754-761e-4f39-8e1e-8b0ad932004d&amp;algo_exp_id=b81f8754-761e-4f39-8e1e-8b0ad932004d-1&amp;pdp_ext_f=%7B%22order%22%3A%229715%22%2C%22eval%22%3A%221%22%2C%22orig_sl_item_id%22%3A%221005006967374887%22%2C%22orig_item_id%22%3A%221005009890367599%22%2C%22fromPage%22%3A%22search%22%7D&amp;pdp_npi=6%40dis%21EUR%213.25%213.26%21%21%2124.77%2124.77%21%400be71e1e17891329941181728e0d20%2112000038886039687%21sea%21LU%210%21ABX%211%210%21n_tag%3A-29910%3Bd%3Ae8fc6401%3Bm03_new_user%3A-29895&amp;curPageLogUid=rfpOWpE811mR&amp;utparam-url=scene%3Asearch%7Cquery_from%3A%7Cx_object_id%3A1005006967374887%7C_p_origin_prod%3A1005009890367599</t>
+  </si>
+  <si>
+    <t>TENSTAR RP2040 Pro Micro Development Board 16MB</t>
+  </si>
+  <si>
+    <t>Screw-in scabilizers</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Aptos Narrow"/>
       <family val="2"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
+      <name val="Roboto"/>
+      <charset val="238"/>
     </font>
   </fonts>
   <fills count="2">
@@ -167,8 +182,9 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -511,7 +527,7 @@
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="29.140625" customWidth="1"/>
-    <col min="3" max="3" width="19" customWidth="1"/>
+    <col min="3" max="3" width="29.42578125" customWidth="1"/>
     <col min="4" max="4" width="16.5703125" customWidth="1"/>
     <col min="5" max="5" width="15.5703125" customWidth="1"/>
     <col min="6" max="6" width="17.140625" customWidth="1"/>
@@ -529,7 +545,7 @@
         <v>2</v>
       </c>
       <c r="D1" t="s">
-        <v>29</v>
+        <v>26</v>
       </c>
       <c r="E1" t="s">
         <v>3</v>
@@ -575,7 +591,7 @@
         <v>2</v>
       </c>
       <c r="B3" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="D3">
         <v>80</v>
@@ -589,7 +605,7 @@
         <v>3</v>
       </c>
       <c r="B4" t="s">
-        <v>21</v>
+        <v>18</v>
       </c>
       <c r="D4">
         <v>80</v>
@@ -674,11 +690,8 @@
       <c r="A8">
         <v>7</v>
       </c>
-      <c r="B8" t="s">
-        <v>18</v>
-      </c>
-      <c r="C8" t="s">
-        <v>19</v>
+      <c r="B8" s="1" t="s">
+        <v>32</v>
       </c>
       <c r="D8">
         <v>1</v>
@@ -687,10 +700,10 @@
         <v>1</v>
       </c>
       <c r="F8">
-        <v>3.36</v>
+        <v>3.61</v>
       </c>
       <c r="G8" t="s">
-        <v>17</v>
+        <v>31</v>
       </c>
       <c r="H8" t="s">
         <v>6</v>
@@ -701,19 +714,22 @@
         <v>8</v>
       </c>
       <c r="B9" t="s">
+        <v>19</v>
+      </c>
+      <c r="C9" t="s">
+        <v>33</v>
+      </c>
+      <c r="D9" t="s">
+        <v>27</v>
+      </c>
+      <c r="E9" t="s">
+        <v>20</v>
+      </c>
+      <c r="F9" t="s">
         <v>22</v>
       </c>
-      <c r="D9" t="s">
-        <v>30</v>
-      </c>
-      <c r="E9" t="s">
-        <v>23</v>
-      </c>
-      <c r="F9" t="s">
-        <v>25</v>
-      </c>
       <c r="G9" t="s">
-        <v>24</v>
+        <v>21</v>
       </c>
       <c r="H9" t="s">
         <v>6</v>
@@ -724,10 +740,10 @@
         <v>9</v>
       </c>
       <c r="B10" t="s">
-        <v>28</v>
+        <v>25</v>
       </c>
       <c r="C10" t="s">
-        <v>27</v>
+        <v>24</v>
       </c>
       <c r="D10">
         <v>1</v>
@@ -735,8 +751,11 @@
       <c r="E10">
         <v>10</v>
       </c>
+      <c r="F10">
+        <v>2.62</v>
+      </c>
       <c r="G10" t="s">
-        <v>26</v>
+        <v>23</v>
       </c>
       <c r="H10" t="s">
         <v>6</v>
@@ -745,6 +764,24 @@
     <row r="11" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A11">
         <v>10</v>
+      </c>
+      <c r="B11" t="s">
+        <v>28</v>
+      </c>
+      <c r="C11" t="s">
+        <v>30</v>
+      </c>
+      <c r="D11">
+        <v>1</v>
+      </c>
+      <c r="E11">
+        <v>1</v>
+      </c>
+      <c r="F11">
+        <v>1.92</v>
+      </c>
+      <c r="G11" t="s">
+        <v>29</v>
       </c>
       <c r="H11" t="s">
         <v>6</v>

</xml_diff>